<commit_message>
NPB自動更新(1軍): 2026-09-24 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-24.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-24.xlsx
@@ -34592,7 +34592,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9回2安打9奪三振の完封勝利で、相手打線を完全に封じ込めた。</t>
+          <t>9回を投げ被安打2、9奪三振の圧巻のピッチングで完封勝利を飾った。</t>
         </is>
       </c>
     </row>
@@ -34607,17 +34607,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>西舘 勇陽</t>
+          <t>坂倉 将吾</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5.1回を投げ10奪三振を奪う力投。失点はあるが、その奪三振能力は際立った。</t>
+          <t>4回裏にランナーを置いて先制2ランホームランを放ち、チームに貴重なリードをもたらした。</t>
         </is>
       </c>
     </row>
@@ -34632,17 +34632,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>坂倉 将吾</t>
+          <t>ダルベック</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>4回裏に先制2ランホームランを放ち、チームに貴重な先制点をもたらした。</t>
+          <t>6回表に右中間へソロホームランを放ち、2点差を1点差に詰め寄る一打となった。</t>
         </is>
       </c>
     </row>
@@ -34657,7 +34657,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ダルベック</t>
+          <t>西舘 勇陽</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -34667,7 +34667,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>6回表にソロホームランを放ち、1点差に詰め寄る一打で反撃の狼煙を上げた。</t>
+          <t>5.1回を投げ10奪三振を奪う力投を見せたが、味方の援護なく降板した。</t>
         </is>
       </c>
     </row>
@@ -34682,17 +34682,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>勝田 成</t>
+          <t>達 孝太</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>広島</t>
+          <t>楽天</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>6回裏にタイムリーヒットを放ち、リードを広げる貴重な決勝打となった。</t>
+          <t>7.1回を投げ2失点と試合を作り、チームの勝利に大きく貢献する好投を見せた。</t>
         </is>
       </c>
     </row>
@@ -34717,7 +34717,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6回1失点の好投で試合を作り、チームの勝利に大きく貢献した。</t>
+          <t>6回を投げ1失点と試合を作り、相手打線を抑え込む安定したピッチングを披露した。</t>
         </is>
       </c>
     </row>

</xml_diff>